<commit_message>
NPB自動更新(1軍): 2026-10-04 (steps: all)
</commit_message>
<xml_diff>
--- a/data/プロ野球/2026年/1軍/レギュラーシーズン/games/datamart/2026-10-04.xlsx
+++ b/data/プロ野球/2026年/1軍/レギュラーシーズン/games/datamart/2026-10-04.xlsx
@@ -75871,7 +75871,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>4回に逆転2ラン、6回にソロと2本塁打を放ち、チームの全得点に絡む活躍を見せた。</t>
+          <t>4回に逆転2ラン、6回にソロを放ち、1試合2本塁打でチームの勝利に大きく貢献した。</t>
         </is>
       </c>
     </row>
@@ -75896,7 +75896,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>延長11回裏、ランナー一二塁のチャンスでライトへのサヨナラヒットを放ち、劇的な勝利を呼び込んだ。</t>
+          <t>延長11回裏、ランナー一二塁からライトへのサヨナラヒットを放ち、劇的な勝利を呼び込んだ。</t>
         </is>
       </c>
     </row>
@@ -75921,7 +75921,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>8回表2アウト満塁の場面で同点タイムリーヒットを放ち、さらに猛打賞も記録した。</t>
+          <t>8回表に同点タイムリーを放ち、さらに4安打猛打賞を記録。打撃でチームを牽引した。</t>
         </is>
       </c>
     </row>
@@ -75946,7 +75946,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>9回表1アウト満塁からライトへのタイムリーヒットで勝ち越し点を挙げ、チームの勝利に貢献した。</t>
+          <t>9回表1死満塁のチャンスで勝ち越しタイムリーを放ち、チームの逆転勝利に貢献した。</t>
         </is>
       </c>
     </row>
@@ -75961,17 +75961,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>小島 和哉</t>
+          <t>松下 歩叶</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>ロッテ</t>
+          <t>ヤクルト</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>7回を投げ被安打6、1失点と好投。相手先発との投手戦を制し、チームを勝利に導いた。</t>
+          <t>4回裏にレフトスタンドへ3ランホームランを放ち、チームの先制点とリードを広げる活躍を見せた。</t>
         </is>
       </c>
     </row>
@@ -75986,17 +75986,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>平良 拳太郎</t>
+          <t>小島 和哉</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>DeNA</t>
+          <t>ロッテ</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>6回を投げ被安打2、1失点と試合を作り、チームのサヨナラ勝利を呼び込む好投を見せた。</t>
+          <t>7回を投げ被安打6、1失点の好投。粘り強いピッチングで試合を作り、勝利投手となった。</t>
         </is>
       </c>
     </row>

</xml_diff>